<commit_message>
nagar estimate hume pipe and ukhu kheti final
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/वडा बजेट estimate/ukhu kheti/ukhu kheti.xlsx
+++ b/बजेट माग estimate/वडा बजेट estimate/ukhu kheti/ukhu kheti.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8FAAD9F-8893-4C7D-804F-75C2FAB8D90D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20736" windowHeight="11040"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="estimate" sheetId="12" r:id="rId1"/>
@@ -36,10 +37,10 @@
     <definedName name="description_781">#REF!</definedName>
     <definedName name="description_783">[1]Abstract!$B$301</definedName>
     <definedName name="description_784">[3]Abstract!$B$300</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">estimate!$A$1:$K$71</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">estimate!$A$1:$K$70</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">estimate!$1:$8</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -57,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="63">
   <si>
     <t>Government of Nepal</t>
   </si>
@@ -194,9 +195,6 @@
     <t>-13% VAT for bitumen washer</t>
   </si>
   <si>
-    <t>)=$! dL=dL=afSnf] sf]?u]6]8 /+lug ss{6 kftfsf] 5fgf 5fpg] sfd</t>
-  </si>
-  <si>
     <t>-Masonary wall</t>
   </si>
   <si>
@@ -231,9 +229,6 @@
   </si>
   <si>
     <t>-deduction for tunnel</t>
-  </si>
-  <si>
-    <t>Provisional sum for unforseen works</t>
   </si>
   <si>
     <t>-MS square pipe of 3" * 3" of 2mm thickness for vertical post</t>
@@ -259,14 +254,17 @@
   <si>
     <t>Date:2082/09/13</t>
   </si>
+  <si>
+    <t>).#^ lblv ).$ dL.dL.afSnf] sf]?u]6]8 /+lug ss{6 kftfsf] 5fgf 5fpg] sfd</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="14" x14ac:knownFonts="1">
     <font>
@@ -425,9 +423,9 @@
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
@@ -439,7 +437,7 @@
     <xf numFmtId="1" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -463,14 +461,14 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="43" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -489,7 +487,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -504,7 +502,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -535,29 +533,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -578,17 +561,32 @@
     <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Comma 2" xfId="3"/>
+    <cellStyle name="Comma 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="2"/>
-    <cellStyle name="Normal 3" xfId="5"/>
-    <cellStyle name="Percent 2" xfId="4"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
+    <cellStyle name="Normal 3" xfId="5" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="Percent 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -604,7 +602,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -698,7 +696,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -757,7 +755,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -821,9 +819,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -861,9 +859,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -898,7 +896,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -933,7 +931,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1106,135 +1104,135 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S71"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:S70"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.6640625" style="19" customWidth="1"/>
-    <col min="2" max="2" width="30.88671875" style="19" customWidth="1"/>
-    <col min="3" max="3" width="4.44140625" style="19" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.44140625" style="19" customWidth="1"/>
-    <col min="5" max="5" width="8.5546875" style="19" customWidth="1"/>
-    <col min="6" max="6" width="7.33203125" style="19" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" style="19"/>
+    <col min="1" max="1" width="4.7109375" style="19" customWidth="1"/>
+    <col min="2" max="2" width="30.85546875" style="19" customWidth="1"/>
+    <col min="3" max="3" width="4.42578125" style="19" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.42578125" style="19" customWidth="1"/>
+    <col min="5" max="5" width="8.5703125" style="19" customWidth="1"/>
+    <col min="6" max="6" width="7.28515625" style="19" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" style="19"/>
     <col min="8" max="8" width="5" style="19" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.5546875" style="19" customWidth="1"/>
-    <col min="10" max="10" width="10.6640625" style="19" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="9.109375" style="19"/>
+    <col min="9" max="9" width="9.5703125" style="19" customWidth="1"/>
+    <col min="10" max="10" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="9.140625" style="19"/>
     <col min="13" max="16" width="0" style="19" hidden="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.109375" style="19"/>
+    <col min="17" max="16384" width="9.140625" style="19"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1" s="53" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="45"/>
-      <c r="I1" s="45"/>
-      <c r="J1" s="45"/>
-      <c r="K1" s="45"/>
-    </row>
-    <row r="2" spans="1:18" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="46" t="s">
+      <c r="B1" s="53"/>
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
+      <c r="F1" s="53"/>
+      <c r="G1" s="53"/>
+      <c r="H1" s="53"/>
+      <c r="I1" s="53"/>
+      <c r="J1" s="53"/>
+      <c r="K1" s="53"/>
+    </row>
+    <row r="2" spans="1:18" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="54" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A3" s="47" t="s">
+      <c r="B2" s="54"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
+      <c r="I2" s="54"/>
+      <c r="J2" s="54"/>
+      <c r="K2" s="54"/>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A3" s="55" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="47"/>
-      <c r="C3" s="47"/>
-      <c r="D3" s="47"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="47"/>
-      <c r="G3" s="47"/>
-      <c r="H3" s="47"/>
-      <c r="I3" s="47"/>
-      <c r="J3" s="47"/>
-      <c r="K3" s="47"/>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A4" s="47" t="s">
+      <c r="B3" s="55"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="55"/>
+      <c r="H3" s="55"/>
+      <c r="I3" s="55"/>
+      <c r="J3" s="55"/>
+      <c r="K3" s="55"/>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A4" s="55" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="47"/>
-      <c r="C4" s="47"/>
-      <c r="D4" s="47"/>
-      <c r="E4" s="47"/>
-      <c r="F4" s="47"/>
-      <c r="G4" s="47"/>
-      <c r="H4" s="47"/>
-      <c r="I4" s="47"/>
-      <c r="J4" s="47"/>
-      <c r="K4" s="47"/>
-    </row>
-    <row r="5" spans="1:18" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A5" s="48" t="s">
+      <c r="B4" s="55"/>
+      <c r="C4" s="55"/>
+      <c r="D4" s="55"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="55"/>
+      <c r="G4" s="55"/>
+      <c r="H4" s="55"/>
+      <c r="I4" s="55"/>
+      <c r="J4" s="55"/>
+      <c r="K4" s="55"/>
+    </row>
+    <row r="5" spans="1:18" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A5" s="56" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="48"/>
-      <c r="C5" s="48"/>
-      <c r="D5" s="48"/>
-      <c r="E5" s="48"/>
-      <c r="F5" s="48"/>
-      <c r="G5" s="48"/>
-      <c r="H5" s="48"/>
-      <c r="I5" s="48"/>
-      <c r="J5" s="48"/>
-      <c r="K5" s="48"/>
-    </row>
-    <row r="6" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="43" t="s">
-        <v>62</v>
-      </c>
-      <c r="B6" s="43"/>
-      <c r="C6" s="43"/>
-      <c r="D6" s="43"/>
-      <c r="E6" s="43"/>
-      <c r="F6" s="43"/>
+      <c r="B5" s="56"/>
+      <c r="C5" s="56"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="56"/>
+      <c r="F5" s="56"/>
+      <c r="G5" s="56"/>
+      <c r="H5" s="56"/>
+      <c r="I5" s="56"/>
+      <c r="J5" s="56"/>
+      <c r="K5" s="56"/>
+    </row>
+    <row r="6" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="51" t="s">
+        <v>60</v>
+      </c>
+      <c r="B6" s="51"/>
+      <c r="C6" s="51"/>
+      <c r="D6" s="51"/>
+      <c r="E6" s="51"/>
+      <c r="F6" s="51"/>
       <c r="G6" s="10"/>
-      <c r="H6" s="44" t="s">
+      <c r="H6" s="52" t="s">
         <v>25</v>
       </c>
-      <c r="I6" s="44"/>
-      <c r="J6" s="44"/>
-      <c r="K6" s="44"/>
-    </row>
-    <row r="7" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="51" t="s">
-        <v>49</v>
-      </c>
-      <c r="B7" s="51"/>
-      <c r="C7" s="51"/>
-      <c r="D7" s="51"/>
-      <c r="E7" s="51"/>
-      <c r="F7" s="51"/>
+      <c r="I6" s="52"/>
+      <c r="J6" s="52"/>
+      <c r="K6" s="52"/>
+    </row>
+    <row r="7" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="46" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="46"/>
+      <c r="C7" s="46"/>
+      <c r="D7" s="46"/>
+      <c r="E7" s="46"/>
+      <c r="F7" s="46"/>
       <c r="G7" s="11"/>
-      <c r="H7" s="52" t="s">
-        <v>63</v>
-      </c>
-      <c r="I7" s="52"/>
-      <c r="J7" s="52"/>
-      <c r="K7" s="52"/>
-    </row>
-    <row r="8" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H7" s="47" t="s">
+        <v>61</v>
+      </c>
+      <c r="I7" s="47"/>
+      <c r="J7" s="47"/>
+      <c r="K7" s="47"/>
+    </row>
+    <row r="8" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
         <v>5</v>
       </c>
@@ -1269,7 +1267,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:18" s="35" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" s="35" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>1</v>
       </c>
@@ -1294,217 +1292,238 @@
       <c r="J9" s="39"/>
       <c r="K9" s="5"/>
     </row>
-    <row r="10" spans="1:18" s="35" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" s="35" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="16"/>
       <c r="B10" s="40" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C10" s="41">
-        <f>2*2</f>
-        <v>4</v>
+        <f>2*3</f>
+        <v>6</v>
       </c>
       <c r="D10" s="9">
-        <f>(10+1+2)/3.281</f>
-        <v>3.9622066443157573</v>
+        <f>(11+1+2)/3.281</f>
+        <v>4.2669917708015843</v>
       </c>
       <c r="E10" s="9">
         <v>4.4000000000000004</v>
       </c>
       <c r="F10" s="9">
-        <f t="shared" ref="F10:F12" si="0">PRODUCT(C10:E10)</f>
-        <v>69.734836939957333</v>
+        <f t="shared" ref="F10:F14" si="0">PRODUCT(C10:E10)</f>
+        <v>112.64858274916183</v>
       </c>
       <c r="G10" s="9">
-        <f t="shared" ref="G10:G12" si="1">F10</f>
-        <v>69.734836939957333</v>
+        <f t="shared" ref="G10:G14" si="1">F10</f>
+        <v>112.64858274916183</v>
       </c>
       <c r="H10" s="39"/>
       <c r="I10" s="39"/>
       <c r="J10" s="39"/>
       <c r="K10" s="27"/>
     </row>
-    <row r="11" spans="1:18" s="35" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="16"/>
       <c r="B11" s="40"/>
       <c r="C11" s="41">
-        <f>2*2</f>
-        <v>4</v>
+        <f>2*3</f>
+        <v>6</v>
       </c>
       <c r="D11" s="9">
-        <f>(10+1+1+2)/3.281</f>
-        <v>4.2669917708015843</v>
+        <f>(11+1+1+2)/3.281</f>
+        <v>4.5717768972874122</v>
       </c>
       <c r="E11" s="9">
         <v>4.4000000000000004</v>
       </c>
       <c r="F11" s="9">
-        <f t="shared" ref="F11" si="2">PRODUCT(C11:E11)</f>
-        <v>75.099055166107888</v>
+        <f t="shared" ref="F11:F12" si="2">PRODUCT(C11:E11)</f>
+        <v>120.69491008838769</v>
       </c>
       <c r="G11" s="9">
-        <f t="shared" ref="G11" si="3">F11</f>
-        <v>75.099055166107888</v>
+        <f t="shared" ref="G11:G12" si="3">F11</f>
+        <v>120.69491008838769</v>
       </c>
       <c r="H11" s="39"/>
       <c r="I11" s="39"/>
       <c r="J11" s="39"/>
       <c r="K11" s="27"/>
     </row>
-    <row r="12" spans="1:18" s="35" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="16"/>
-      <c r="B12" s="40" t="s">
-        <v>60</v>
-      </c>
+      <c r="B12" s="40"/>
       <c r="C12" s="41">
-        <f>2*(2+1)</f>
-        <v>6</v>
+        <f>2</f>
+        <v>2</v>
       </c>
       <c r="D12" s="9">
-        <f>(12+3)/3.281</f>
-        <v>4.5717768972874122</v>
+        <f>(11+1+2)/3.281</f>
+        <v>4.2669917708015843</v>
       </c>
       <c r="E12" s="9">
-        <v>3.01</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="F12" s="9">
-        <f t="shared" si="0"/>
-        <v>82.566290765010663</v>
+        <f t="shared" si="2"/>
+        <v>37.549527583053944</v>
       </c>
       <c r="G12" s="9">
-        <f t="shared" si="1"/>
-        <v>82.566290765010663</v>
+        <f t="shared" si="3"/>
+        <v>37.549527583053944</v>
       </c>
       <c r="H12" s="39"/>
       <c r="I12" s="39"/>
       <c r="J12" s="39"/>
       <c r="K12" s="27"/>
-      <c r="Q12" s="35">
-        <f>PRODUCT(C12:D12)</f>
-        <v>27.430661383724473</v>
-      </c>
-      <c r="R12" s="35">
-        <f>CONVERT(Q12,"m","ft")</f>
-        <v>89.995608214319134</v>
-      </c>
-    </row>
-    <row r="13" spans="1:18" s="35" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:18" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="16"/>
       <c r="B13" s="40"/>
       <c r="C13" s="41">
-        <f>2*(2+1)</f>
-        <v>6</v>
+        <f>2</f>
+        <v>2</v>
       </c>
       <c r="D13" s="9">
-        <f>(10+3)/3.281</f>
-        <v>3.9622066443157573</v>
+        <f>(11+1+1+2)/3.281</f>
+        <v>4.5717768972874122</v>
       </c>
       <c r="E13" s="9">
-        <v>3.01</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="F13" s="9">
         <f t="shared" ref="F13" si="4">PRODUCT(C13:E13)</f>
-        <v>71.557451996342579</v>
+        <v>40.231636696129229</v>
       </c>
       <c r="G13" s="9">
         <f t="shared" ref="G13" si="5">F13</f>
-        <v>71.557451996342579</v>
+        <v>40.231636696129229</v>
       </c>
       <c r="H13" s="39"/>
       <c r="I13" s="39"/>
       <c r="J13" s="39"/>
       <c r="K13" s="27"/>
     </row>
-    <row r="14" spans="1:18" s="35" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" s="35" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="16"/>
       <c r="B14" s="40" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C14" s="41">
-        <f>2*2</f>
-        <v>4</v>
+        <f>2*(2+1)</f>
+        <v>6</v>
       </c>
       <c r="D14" s="9">
         <f>(12+3)/3.281</f>
         <v>4.5717768972874122</v>
       </c>
       <c r="E14" s="9">
-        <v>2.2599999999999998</v>
+        <v>3.01</v>
       </c>
       <c r="F14" s="9">
-        <f t="shared" ref="F14" si="6">PRODUCT(C14:E14)</f>
-        <v>41.328863151478203</v>
+        <f t="shared" si="0"/>
+        <v>82.566290765010663</v>
       </c>
       <c r="G14" s="9">
-        <f t="shared" ref="G14" si="7">F14</f>
-        <v>41.328863151478203</v>
+        <f t="shared" si="1"/>
+        <v>82.566290765010663</v>
       </c>
       <c r="H14" s="39"/>
       <c r="I14" s="39"/>
       <c r="J14" s="39"/>
       <c r="K14" s="27"/>
-    </row>
-    <row r="15" spans="1:18" s="35" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="2"/>
-      <c r="B15" s="40" t="s">
+      <c r="Q14" s="35">
+        <f>PRODUCT(C14:D14)</f>
+        <v>27.430661383724473</v>
+      </c>
+      <c r="R14" s="35">
+        <f>CONVERT(Q14,"m","ft")</f>
+        <v>89.995608214319134</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" s="35" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="16"/>
+      <c r="B15" s="40"/>
+      <c r="C15" s="41">
+        <f>2*(2+1)</f>
+        <v>6</v>
+      </c>
+      <c r="D15" s="9">
+        <f>(10+3)/3.281</f>
+        <v>3.9622066443157573</v>
+      </c>
+      <c r="E15" s="9">
+        <v>3.01</v>
+      </c>
+      <c r="F15" s="9">
+        <f t="shared" ref="F15" si="6">PRODUCT(C15:E15)</f>
+        <v>71.557451996342579</v>
+      </c>
+      <c r="G15" s="9">
+        <f t="shared" ref="G15" si="7">F15</f>
+        <v>71.557451996342579</v>
+      </c>
+      <c r="H15" s="39"/>
+      <c r="I15" s="39"/>
+      <c r="J15" s="39"/>
+      <c r="K15" s="27"/>
+    </row>
+    <row r="16" spans="1:18" s="35" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A16" s="16"/>
+      <c r="B16" s="40" t="s">
+        <v>59</v>
+      </c>
+      <c r="C16" s="41">
+        <f>2*2</f>
+        <v>4</v>
+      </c>
+      <c r="D16" s="9">
+        <f>(12+3)/3.281</f>
+        <v>4.5717768972874122</v>
+      </c>
+      <c r="E16" s="9">
+        <v>2.2599999999999998</v>
+      </c>
+      <c r="F16" s="9">
+        <f t="shared" ref="F16" si="8">PRODUCT(C16:E16)</f>
+        <v>41.328863151478203</v>
+      </c>
+      <c r="G16" s="9">
+        <f t="shared" ref="G16" si="9">F16</f>
+        <v>41.328863151478203</v>
+      </c>
+      <c r="H16" s="39"/>
+      <c r="I16" s="39"/>
+      <c r="J16" s="39"/>
+      <c r="K16" s="27"/>
+    </row>
+    <row r="17" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2"/>
+      <c r="B17" s="40" t="s">
         <v>36</v>
       </c>
-      <c r="C15" s="3"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="39">
-        <f>SUM(G10:G14)</f>
-        <v>340.28649801889662</v>
-      </c>
-      <c r="H15" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="I15" s="6">
-        <v>182.51</v>
-      </c>
-      <c r="J15" s="39">
-        <f>G15*I15</f>
-        <v>62105.688753428818</v>
-      </c>
-      <c r="K15" s="5"/>
-    </row>
-    <row r="16" spans="1:18" s="35" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="2"/>
-      <c r="B16" s="40" t="s">
-        <v>38</v>
-      </c>
-      <c r="C16" s="3"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="39"/>
-      <c r="H16" s="7"/>
-      <c r="I16" s="6"/>
-      <c r="J16" s="39">
-        <f>0.13*G15*(1871.42/18.94)</f>
-        <v>4370.985457018377</v>
-      </c>
-      <c r="K16" s="5"/>
-    </row>
-    <row r="17" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="2"/>
-      <c r="B17" s="40"/>
       <c r="C17" s="3"/>
       <c r="D17" s="4"/>
       <c r="E17" s="5"/>
       <c r="F17" s="5"/>
-      <c r="G17" s="39"/>
-      <c r="H17" s="7"/>
-      <c r="I17" s="6"/>
-      <c r="J17" s="39"/>
+      <c r="G17" s="39">
+        <f>SUM(G10:G16)</f>
+        <v>506.57726302956416</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="I17" s="6">
+        <v>182.51</v>
+      </c>
+      <c r="J17" s="39">
+        <f>G17*I17</f>
+        <v>92455.416275525757</v>
+      </c>
       <c r="K17" s="5"/>
     </row>
-    <row r="18" spans="1:11" s="35" customFormat="1" ht="30" x14ac:dyDescent="0.3">
-      <c r="A18" s="2">
-        <v>2</v>
-      </c>
-      <c r="B18" s="36" t="s">
-        <v>45</v>
+    <row r="18" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2"/>
+      <c r="B18" s="40" t="s">
+        <v>38</v>
       </c>
       <c r="C18" s="3"/>
       <c r="D18" s="4"/>
@@ -1513,119 +1532,122 @@
       <c r="G18" s="39"/>
       <c r="H18" s="7"/>
       <c r="I18" s="6"/>
-      <c r="J18" s="39"/>
+      <c r="J18" s="39">
+        <f>0.13*G17*(1871.42/18.94)</f>
+        <v>6506.9929675418325</v>
+      </c>
       <c r="K18" s="5"/>
     </row>
-    <row r="19" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
-      <c r="B19" s="40" t="s">
-        <v>39</v>
-      </c>
-      <c r="C19" s="3">
-        <f>2*1</f>
-        <v>2</v>
-      </c>
-      <c r="D19" s="4">
-        <f>(10+3)/3.281</f>
-        <v>3.9622066443157573</v>
-      </c>
-      <c r="E19" s="5">
-        <f>(12+3)/3.281</f>
-        <v>4.5717768972874122</v>
-      </c>
+      <c r="B19" s="40"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="5"/>
       <c r="F19" s="5"/>
-      <c r="G19" s="33">
-        <f t="shared" ref="G19" si="8">PRODUCT(C19:F19)</f>
-        <v>36.228649597522924</v>
-      </c>
+      <c r="G19" s="39"/>
       <c r="H19" s="7"/>
       <c r="I19" s="6"/>
       <c r="J19" s="39"/>
       <c r="K19" s="5"/>
     </row>
-    <row r="20" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="2"/>
-      <c r="B20" s="40" t="s">
-        <v>36</v>
+    <row r="20" spans="1:11" s="35" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A20" s="2">
+        <v>2</v>
+      </c>
+      <c r="B20" s="36" t="s">
+        <v>62</v>
       </c>
       <c r="C20" s="3"/>
       <c r="D20" s="4"/>
       <c r="E20" s="5"/>
       <c r="F20" s="5"/>
-      <c r="G20" s="39">
-        <f>SUM(G19:G19)</f>
+      <c r="G20" s="39"/>
+      <c r="H20" s="7"/>
+      <c r="I20" s="6"/>
+      <c r="J20" s="39"/>
+      <c r="K20" s="5"/>
+    </row>
+    <row r="21" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="2"/>
+      <c r="B21" s="40" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" s="3">
+        <f>2*1</f>
+        <v>2</v>
+      </c>
+      <c r="D21" s="4">
+        <f>(10+3)/3.281</f>
+        <v>3.9622066443157573</v>
+      </c>
+      <c r="E21" s="5">
+        <f>(12+3)/3.281</f>
+        <v>4.5717768972874122</v>
+      </c>
+      <c r="F21" s="5"/>
+      <c r="G21" s="33">
+        <f t="shared" ref="G21" si="10">PRODUCT(C21:F21)</f>
         <v>36.228649597522924</v>
       </c>
-      <c r="H20" s="7" t="s">
+      <c r="H21" s="7"/>
+      <c r="I21" s="6"/>
+      <c r="J21" s="39"/>
+      <c r="K21" s="5"/>
+    </row>
+    <row r="22" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="2"/>
+      <c r="B22" s="40"/>
+      <c r="C22" s="3">
+        <v>1</v>
+      </c>
+      <c r="D22" s="4">
+        <f>(10+3)/3.281</f>
+        <v>3.9622066443157573</v>
+      </c>
+      <c r="E22" s="5">
+        <f>(10+3)/3.281</f>
+        <v>3.9622066443157573</v>
+      </c>
+      <c r="F22" s="5"/>
+      <c r="G22" s="33">
+        <f t="shared" ref="G22" si="11">PRODUCT(C22:F22)</f>
+        <v>15.699081492259934</v>
+      </c>
+      <c r="H22" s="7"/>
+      <c r="I22" s="6"/>
+      <c r="J22" s="39"/>
+      <c r="K22" s="5"/>
+    </row>
+    <row r="23" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="2"/>
+      <c r="B23" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="C23" s="3"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="39">
+        <f>SUM(G21:G22)</f>
+        <v>51.92773108978286</v>
+      </c>
+      <c r="H23" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="I20" s="6">
-        <v>1112.58</v>
-      </c>
-      <c r="J20" s="39">
-        <f>G20*I20</f>
-        <v>40307.270969212055</v>
-      </c>
-      <c r="K20" s="5"/>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A21" s="16"/>
-      <c r="B21" s="32" t="s">
-        <v>41</v>
-      </c>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="17"/>
-      <c r="G21" s="17"/>
-      <c r="H21" s="17"/>
-      <c r="I21" s="17"/>
-      <c r="J21" s="18">
-        <f>0.13*G20*7050.67/10</f>
-        <v>3320.6712871509708</v>
-      </c>
-      <c r="K21" s="17"/>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A22" s="16"/>
-      <c r="B22" s="32" t="s">
-        <v>42</v>
-      </c>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="17"/>
-      <c r="F22" s="17"/>
-      <c r="G22" s="17"/>
-      <c r="H22" s="17"/>
-      <c r="I22" s="17"/>
-      <c r="J22" s="18">
-        <f>0.13*G20*1023.75/10</f>
-        <v>482.15804033103325</v>
-      </c>
-      <c r="K22" s="17"/>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A23" s="16"/>
-      <c r="B23" s="32" t="s">
-        <v>43</v>
-      </c>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="17"/>
-      <c r="G23" s="17"/>
-      <c r="H23" s="17"/>
-      <c r="I23" s="17"/>
-      <c r="J23" s="18">
-        <f>0.13*G20*348.21/10</f>
-        <v>163.99731499259494</v>
-      </c>
-      <c r="K23" s="17"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="I23" s="6">
+        <v>1074.98</v>
+      </c>
+      <c r="J23" s="39">
+        <f>G23*I23</f>
+        <v>55821.27236689478</v>
+      </c>
+      <c r="K23" s="5"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="16"/>
       <c r="B24" s="32" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C24" s="17"/>
       <c r="D24" s="17"/>
@@ -1635,14 +1657,16 @@
       <c r="H24" s="17"/>
       <c r="I24" s="17"/>
       <c r="J24" s="18">
-        <f>0.13*G20*165/10</f>
-        <v>77.71045338668668</v>
+        <f>0.13*G23*6674.66/10</f>
+        <v>4505.7993447444915</v>
       </c>
       <c r="K24" s="17"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="16"/>
-      <c r="B25" s="32"/>
+      <c r="B25" s="32" t="s">
+        <v>42</v>
+      </c>
       <c r="C25" s="17"/>
       <c r="D25" s="17"/>
       <c r="E25" s="17"/>
@@ -1650,15 +1674,16 @@
       <c r="G25" s="17"/>
       <c r="H25" s="17"/>
       <c r="I25" s="17"/>
-      <c r="J25" s="18"/>
+      <c r="J25" s="18">
+        <f>0.13*G23*1023.75/10</f>
+        <v>691.09319114114771</v>
+      </c>
       <c r="K25" s="17"/>
     </row>
-    <row r="26" spans="1:11" ht="30.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="16">
-        <v>3</v>
-      </c>
-      <c r="B26" s="56" t="s">
-        <v>50</v>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26" s="16"/>
+      <c r="B26" s="32" t="s">
+        <v>43</v>
       </c>
       <c r="C26" s="17"/>
       <c r="D26" s="17"/>
@@ -1667,300 +1692,288 @@
       <c r="G26" s="17"/>
       <c r="H26" s="17"/>
       <c r="I26" s="17"/>
-      <c r="J26" s="18"/>
+      <c r="J26" s="18">
+        <f>0.13*G23*348.21/10</f>
+        <v>235.06281815605274</v>
+      </c>
       <c r="K26" s="17"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="16"/>
       <c r="B27" s="32" t="s">
-        <v>46</v>
-      </c>
-      <c r="C27" s="17">
-        <f>2*2</f>
-        <v>4</v>
-      </c>
-      <c r="D27" s="33">
-        <f>12/3.281</f>
-        <v>3.6574215178299299</v>
-      </c>
-      <c r="E27" s="17">
-        <v>0.45</v>
-      </c>
-      <c r="F27" s="17">
-        <v>0.6</v>
-      </c>
-      <c r="G27" s="33">
-        <f t="shared" ref="G27:G28" si="9">PRODUCT(C27:F27)</f>
-        <v>3.9500152392563241</v>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="17"/>
       <c r="H27" s="17"/>
       <c r="I27" s="17"/>
-      <c r="J27" s="18"/>
+      <c r="J27" s="18">
+        <f>0.13*G23*165/10</f>
+        <v>111.38498318758425</v>
+      </c>
       <c r="K27" s="17"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="16"/>
-      <c r="B28" s="32" t="s">
-        <v>48</v>
-      </c>
-      <c r="C28" s="17">
-        <f>2*4</f>
-        <v>8</v>
-      </c>
-      <c r="D28" s="33">
-        <v>0.6</v>
-      </c>
-      <c r="E28" s="17">
-        <v>0.6</v>
-      </c>
-      <c r="F28" s="17">
-        <v>0.6</v>
-      </c>
-      <c r="G28" s="33">
-        <f t="shared" si="9"/>
-        <v>1.728</v>
-      </c>
+      <c r="B28" s="32"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="17"/>
       <c r="H28" s="17"/>
       <c r="I28" s="17"/>
       <c r="J28" s="18"/>
       <c r="K28" s="17"/>
     </row>
-    <row r="29" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="2"/>
-      <c r="B29" s="40" t="s">
-        <v>36</v>
-      </c>
-      <c r="C29" s="3"/>
-      <c r="D29" s="4"/>
-      <c r="E29" s="5"/>
-      <c r="F29" s="5"/>
-      <c r="G29" s="39">
-        <f>SUM(G27:G28)</f>
-        <v>5.6780152392563243</v>
-      </c>
-      <c r="H29" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="I29" s="6">
-        <v>674.12</v>
-      </c>
-      <c r="J29" s="39">
-        <f>G29*I29</f>
-        <v>3827.6636330874735</v>
-      </c>
-      <c r="K29" s="5"/>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" ht="30.75" x14ac:dyDescent="0.25">
+      <c r="A29" s="16">
+        <v>3</v>
+      </c>
+      <c r="B29" s="43" t="s">
+        <v>49</v>
+      </c>
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="17"/>
+      <c r="H29" s="17"/>
+      <c r="I29" s="17"/>
+      <c r="J29" s="18"/>
+      <c r="K29" s="17"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="16"/>
-      <c r="B30" s="32"/>
-      <c r="C30" s="17"/>
-      <c r="D30" s="17"/>
-      <c r="E30" s="17"/>
-      <c r="F30" s="17"/>
-      <c r="G30" s="17"/>
+      <c r="B30" s="32" t="s">
+        <v>45</v>
+      </c>
+      <c r="C30" s="17">
+        <f>2*2</f>
+        <v>4</v>
+      </c>
+      <c r="D30" s="33">
+        <f>8/3.281</f>
+        <v>2.4382810118866196</v>
+      </c>
+      <c r="E30" s="17">
+        <v>0.45</v>
+      </c>
+      <c r="F30" s="17">
+        <v>0.9</v>
+      </c>
+      <c r="G30" s="33">
+        <f t="shared" ref="G30:G31" si="12">PRODUCT(C30:F30)</f>
+        <v>3.9500152392563237</v>
+      </c>
       <c r="H30" s="17"/>
       <c r="I30" s="17"/>
       <c r="J30" s="18"/>
       <c r="K30" s="17"/>
     </row>
-    <row r="31" spans="1:11" ht="30.6" x14ac:dyDescent="0.3">
-      <c r="A31" s="16">
-        <v>4</v>
-      </c>
-      <c r="B31" s="56" t="s">
-        <v>51</v>
-      </c>
-      <c r="C31" s="17"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="17"/>
-      <c r="F31" s="17"/>
-      <c r="G31" s="17"/>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" s="16"/>
+      <c r="B31" s="32" t="s">
+        <v>47</v>
+      </c>
+      <c r="C31" s="17">
+        <f>2*4</f>
+        <v>8</v>
+      </c>
+      <c r="D31" s="33">
+        <v>0.6</v>
+      </c>
+      <c r="E31" s="17">
+        <v>0.6</v>
+      </c>
+      <c r="F31" s="17">
+        <v>0.6</v>
+      </c>
+      <c r="G31" s="33">
+        <f t="shared" si="12"/>
+        <v>1.728</v>
+      </c>
       <c r="H31" s="17"/>
       <c r="I31" s="17"/>
       <c r="J31" s="18"/>
       <c r="K31" s="17"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A32" s="16"/>
-      <c r="B32" s="32" t="str">
-        <f>B27</f>
-        <v>-Masonary wall</v>
-      </c>
-      <c r="C32" s="17">
-        <f>C27</f>
-        <v>4</v>
-      </c>
-      <c r="D32" s="33">
-        <f>D27</f>
-        <v>3.6574215178299299</v>
-      </c>
-      <c r="E32" s="33">
-        <v>0.45</v>
-      </c>
-      <c r="F32" s="33">
-        <v>0.15</v>
-      </c>
-      <c r="G32" s="33">
-        <f t="shared" ref="G32:G35" si="10">PRODUCT(C32:F32)</f>
-        <v>0.98750380981408103</v>
-      </c>
-      <c r="H32" s="17"/>
-      <c r="I32" s="17"/>
-      <c r="J32" s="18"/>
-      <c r="K32" s="17"/>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="2"/>
+      <c r="B32" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="C32" s="3"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="5"/>
+      <c r="F32" s="5"/>
+      <c r="G32" s="39">
+        <f>SUM(G30:G31)</f>
+        <v>5.6780152392563235</v>
+      </c>
+      <c r="H32" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="I32" s="6">
+        <v>674.12</v>
+      </c>
+      <c r="J32" s="39">
+        <f>G32*I32</f>
+        <v>3827.6636330874726</v>
+      </c>
+      <c r="K32" s="5"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="16"/>
-      <c r="B33" s="32" t="str">
-        <f>B28</f>
-        <v>-for footing of vertical post</v>
-      </c>
-      <c r="C33" s="17">
-        <f>C28</f>
-        <v>8</v>
-      </c>
-      <c r="D33" s="33">
-        <f>D28</f>
-        <v>0.6</v>
-      </c>
-      <c r="E33" s="33">
-        <f>E28</f>
-        <v>0.6</v>
-      </c>
-      <c r="F33" s="33">
-        <v>0.15</v>
-      </c>
-      <c r="G33" s="33">
-        <f t="shared" si="10"/>
-        <v>0.432</v>
-      </c>
+      <c r="B33" s="32"/>
+      <c r="C33" s="17"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="17"/>
+      <c r="G33" s="17"/>
       <c r="H33" s="17"/>
       <c r="I33" s="17"/>
       <c r="J33" s="18"/>
       <c r="K33" s="17"/>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A34" s="16"/>
-      <c r="B34" s="32" t="s">
-        <v>56</v>
-      </c>
-      <c r="C34" s="17">
-        <f>2*1</f>
-        <v>2</v>
-      </c>
-      <c r="D34" s="33">
-        <f>10/3.281</f>
-        <v>3.047851264858275</v>
-      </c>
-      <c r="E34" s="33">
-        <f>12/3.281</f>
-        <v>3.6574215178299299</v>
-      </c>
-      <c r="F34" s="33">
-        <v>0.15</v>
-      </c>
-      <c r="G34" s="33">
-        <f t="shared" si="10"/>
-        <v>3.3441830397713472</v>
-      </c>
+    <row r="34" spans="1:11" ht="30.75" x14ac:dyDescent="0.25">
+      <c r="A34" s="16">
+        <v>4</v>
+      </c>
+      <c r="B34" s="43" t="s">
+        <v>50</v>
+      </c>
+      <c r="C34" s="17"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="17"/>
+      <c r="F34" s="17"/>
+      <c r="G34" s="17"/>
       <c r="H34" s="17"/>
       <c r="I34" s="17"/>
       <c r="J34" s="18"/>
       <c r="K34" s="17"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="16"/>
-      <c r="B35" s="32" t="s">
-        <v>57</v>
+      <c r="B35" s="32" t="str">
+        <f>B31</f>
+        <v>-for footing of vertical post</v>
       </c>
       <c r="C35" s="17">
-        <f>2*-1</f>
-        <v>-2</v>
+        <f>C31</f>
+        <v>8</v>
       </c>
       <c r="D35" s="33">
-        <f>12/3.281</f>
-        <v>3.6574215178299299</v>
+        <f>D31</f>
+        <v>0.6</v>
       </c>
       <c r="E35" s="33">
-        <f>0.6+0.45+0.45</f>
-        <v>1.5</v>
+        <f>E31</f>
+        <v>0.6</v>
       </c>
       <c r="F35" s="33">
         <v>0.15</v>
       </c>
       <c r="G35" s="33">
-        <f t="shared" si="10"/>
-        <v>-1.6458396830234685</v>
+        <f t="shared" ref="G35:G37" si="13">PRODUCT(C35:F35)</f>
+        <v>0.432</v>
       </c>
       <c r="H35" s="17"/>
       <c r="I35" s="17"/>
       <c r="J35" s="18"/>
       <c r="K35" s="17"/>
     </row>
-    <row r="36" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="2"/>
-      <c r="B36" s="40" t="s">
-        <v>36</v>
-      </c>
-      <c r="C36" s="3"/>
-      <c r="D36" s="4"/>
-      <c r="E36" s="5"/>
-      <c r="F36" s="5"/>
-      <c r="G36" s="39">
-        <f>SUM(G32:G35)</f>
-        <v>3.11784716656196</v>
-      </c>
-      <c r="H36" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="I36" s="6">
-        <v>4495.6400000000003</v>
-      </c>
-      <c r="J36" s="39">
-        <f>G36*I36</f>
-        <v>14016.718435882611</v>
-      </c>
-      <c r="K36" s="5"/>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36" s="16"/>
+      <c r="B36" s="32" t="s">
+        <v>55</v>
+      </c>
+      <c r="C36" s="17">
+        <f>2*1</f>
+        <v>2</v>
+      </c>
+      <c r="D36" s="33">
+        <f>10/3.281</f>
+        <v>3.047851264858275</v>
+      </c>
+      <c r="E36" s="33">
+        <f>12/3.281</f>
+        <v>3.6574215178299299</v>
+      </c>
+      <c r="F36" s="33">
+        <v>0.15</v>
+      </c>
+      <c r="G36" s="33">
+        <f t="shared" si="13"/>
+        <v>3.3441830397713472</v>
+      </c>
+      <c r="H36" s="17"/>
+      <c r="I36" s="17"/>
+      <c r="J36" s="18"/>
+      <c r="K36" s="17"/>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="16"/>
       <c r="B37" s="32" t="s">
-        <v>52</v>
-      </c>
-      <c r="C37" s="17"/>
-      <c r="D37" s="17"/>
-      <c r="E37" s="17"/>
-      <c r="F37" s="17"/>
-      <c r="G37" s="17"/>
+        <v>56</v>
+      </c>
+      <c r="C37" s="17">
+        <f>2*-1</f>
+        <v>-2</v>
+      </c>
+      <c r="D37" s="33">
+        <f>8/3.281</f>
+        <v>2.4382810118866196</v>
+      </c>
+      <c r="E37" s="33">
+        <f>0.6+0.45+0.45</f>
+        <v>1.5</v>
+      </c>
+      <c r="F37" s="33">
+        <v>0.15</v>
+      </c>
+      <c r="G37" s="33">
+        <f t="shared" si="13"/>
+        <v>-1.0972264553489788</v>
+      </c>
       <c r="H37" s="17"/>
       <c r="I37" s="17"/>
-      <c r="J37" s="18">
-        <f>0.13*G36*2577.63</f>
-        <v>1044.7653309528637</v>
-      </c>
+      <c r="J37" s="18"/>
       <c r="K37" s="17"/>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A38" s="16"/>
-      <c r="B38" s="32" t="s">
-        <v>53</v>
-      </c>
-      <c r="C38" s="17"/>
-      <c r="D38" s="17"/>
-      <c r="E38" s="17"/>
-      <c r="F38" s="17"/>
-      <c r="G38" s="17"/>
-      <c r="H38" s="17"/>
-      <c r="I38" s="17"/>
-      <c r="J38" s="18">
-        <f>0.13*G36*515.52</f>
-        <v>208.9506342697828</v>
-      </c>
-      <c r="K38" s="17"/>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="2"/>
+      <c r="B38" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="C38" s="3"/>
+      <c r="D38" s="4"/>
+      <c r="E38" s="5"/>
+      <c r="F38" s="5"/>
+      <c r="G38" s="39">
+        <f>SUM(G35:G37)</f>
+        <v>2.6789565844223686</v>
+      </c>
+      <c r="H38" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="I38" s="6">
+        <v>4495.6400000000003</v>
+      </c>
+      <c r="J38" s="39">
+        <f>G38*I38</f>
+        <v>12043.624379192579</v>
+      </c>
+      <c r="K38" s="5"/>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="16"/>
-      <c r="B39" s="42"/>
+      <c r="B39" s="32" t="s">
+        <v>51</v>
+      </c>
       <c r="C39" s="17"/>
       <c r="D39" s="17"/>
       <c r="E39" s="17"/>
@@ -1968,15 +1981,16 @@
       <c r="G39" s="17"/>
       <c r="H39" s="17"/>
       <c r="I39" s="17"/>
-      <c r="J39" s="18"/>
+      <c r="J39" s="18">
+        <f>0.13*G38*2577.63</f>
+        <v>897.69665189160207</v>
+      </c>
       <c r="K39" s="17"/>
     </row>
-    <row r="40" spans="1:11" ht="30.6" x14ac:dyDescent="0.3">
-      <c r="A40" s="16">
-        <v>5</v>
-      </c>
-      <c r="B40" s="56" t="s">
-        <v>54</v>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A40" s="16"/>
+      <c r="B40" s="32" t="s">
+        <v>52</v>
       </c>
       <c r="C40" s="17"/>
       <c r="D40" s="17"/>
@@ -1985,196 +1999,183 @@
       <c r="G40" s="17"/>
       <c r="H40" s="17"/>
       <c r="I40" s="17"/>
-      <c r="J40" s="17"/>
+      <c r="J40" s="18">
+        <f>0.13*G38*515.52</f>
+        <v>179.53724079218455</v>
+      </c>
       <c r="K40" s="17"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="16"/>
-      <c r="B41" s="32" t="s">
-        <v>46</v>
-      </c>
-      <c r="C41" s="17">
-        <f>C32</f>
-        <v>4</v>
-      </c>
-      <c r="D41" s="33">
-        <f>D32</f>
-        <v>3.6574215178299299</v>
-      </c>
-      <c r="E41" s="33">
-        <v>0.45</v>
-      </c>
-      <c r="F41" s="17">
-        <v>0.05</v>
-      </c>
-      <c r="G41" s="33">
-        <f t="shared" ref="G41:G42" si="11">PRODUCT(C41:F41)</f>
-        <v>0.32916793660469373</v>
-      </c>
+      <c r="B41" s="42"/>
+      <c r="C41" s="17"/>
+      <c r="D41" s="17"/>
+      <c r="E41" s="17"/>
+      <c r="F41" s="17"/>
+      <c r="G41" s="17"/>
       <c r="H41" s="17"/>
       <c r="I41" s="17"/>
       <c r="J41" s="18"/>
       <c r="K41" s="17"/>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A42" s="16"/>
-      <c r="B42" s="32" t="str">
-        <f>B33</f>
-        <v>-for footing of vertical post</v>
-      </c>
-      <c r="C42" s="17">
-        <f>2*4</f>
-        <v>8</v>
-      </c>
-      <c r="D42" s="33">
-        <v>0.6</v>
-      </c>
-      <c r="E42" s="17">
-        <v>0.6</v>
-      </c>
-      <c r="F42" s="33">
-        <v>7.4999999999999997E-2</v>
-      </c>
-      <c r="G42" s="33">
-        <f t="shared" si="11"/>
-        <v>0.216</v>
-      </c>
+    <row r="42" spans="1:11" ht="30.75" x14ac:dyDescent="0.25">
+      <c r="A42" s="16">
+        <v>5</v>
+      </c>
+      <c r="B42" s="43" t="s">
+        <v>53</v>
+      </c>
+      <c r="C42" s="17"/>
+      <c r="D42" s="17"/>
+      <c r="E42" s="17"/>
+      <c r="F42" s="17"/>
+      <c r="G42" s="17"/>
       <c r="H42" s="17"/>
       <c r="I42" s="17"/>
-      <c r="J42" s="18"/>
+      <c r="J42" s="17"/>
       <c r="K42" s="17"/>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="16"/>
-      <c r="B43" s="32"/>
+      <c r="B43" s="32" t="str">
+        <f>B35</f>
+        <v>-for footing of vertical post</v>
+      </c>
       <c r="C43" s="17">
         <f>2*4</f>
         <v>8</v>
       </c>
       <c r="D43" s="33">
-        <v>0.45</v>
+        <v>0.6</v>
       </c>
       <c r="E43" s="17">
-        <v>0.45</v>
+        <v>0.6</v>
       </c>
       <c r="F43" s="33">
-        <v>0.45</v>
+        <v>7.4999999999999997E-2</v>
       </c>
       <c r="G43" s="33">
-        <f t="shared" ref="G43:G45" si="12">PRODUCT(C43:F43)</f>
-        <v>0.72900000000000009</v>
+        <f t="shared" ref="G43" si="14">PRODUCT(C43:F43)</f>
+        <v>0.216</v>
       </c>
       <c r="H43" s="17"/>
       <c r="I43" s="17"/>
       <c r="J43" s="18"/>
       <c r="K43" s="17"/>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="16"/>
-      <c r="B44" s="32" t="str">
-        <f>B34</f>
-        <v>-for flooring</v>
-      </c>
+      <c r="B44" s="32"/>
       <c r="C44" s="17">
-        <f>C34</f>
-        <v>2</v>
+        <f>2*4</f>
+        <v>8</v>
       </c>
       <c r="D44" s="33">
-        <f>D34</f>
-        <v>3.047851264858275</v>
-      </c>
-      <c r="E44" s="33">
-        <f>E34</f>
-        <v>3.6574215178299299</v>
+        <v>0.45</v>
+      </c>
+      <c r="E44" s="17">
+        <v>0.45</v>
       </c>
       <c r="F44" s="33">
-        <v>0.1</v>
+        <v>0.45</v>
       </c>
       <c r="G44" s="33">
-        <f t="shared" si="12"/>
-        <v>2.2294553598475648</v>
+        <f t="shared" ref="G44:G46" si="15">PRODUCT(C44:F44)</f>
+        <v>0.72900000000000009</v>
       </c>
       <c r="H44" s="17"/>
       <c r="I44" s="17"/>
       <c r="J44" s="18"/>
       <c r="K44" s="17"/>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="16"/>
-      <c r="B45" s="32" t="s">
-        <v>57</v>
+      <c r="B45" s="32" t="str">
+        <f>B36</f>
+        <v>-for flooring</v>
       </c>
       <c r="C45" s="17">
-        <f>C35</f>
-        <v>-2</v>
+        <f>C36</f>
+        <v>2</v>
       </c>
       <c r="D45" s="33">
-        <f>12/3.281</f>
+        <f>D36</f>
+        <v>3.047851264858275</v>
+      </c>
+      <c r="E45" s="33">
+        <f>E36</f>
         <v>3.6574215178299299</v>
-      </c>
-      <c r="E45" s="33">
-        <f>0.6+0.45+0.45</f>
-        <v>1.5</v>
       </c>
       <c r="F45" s="33">
         <v>0.1</v>
       </c>
       <c r="G45" s="33">
-        <f t="shared" si="12"/>
-        <v>-1.097226455348979</v>
+        <f t="shared" si="15"/>
+        <v>2.2294553598475648</v>
       </c>
       <c r="H45" s="17"/>
       <c r="I45" s="17"/>
       <c r="J45" s="18"/>
       <c r="K45" s="17"/>
     </row>
-    <row r="46" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="2"/>
-      <c r="B46" s="40" t="s">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A46" s="16"/>
+      <c r="B46" s="32" t="s">
+        <v>56</v>
+      </c>
+      <c r="C46" s="17">
+        <f>C37</f>
+        <v>-2</v>
+      </c>
+      <c r="D46" s="33">
+        <f>12/3.281</f>
+        <v>3.6574215178299299</v>
+      </c>
+      <c r="E46" s="33">
+        <f>0.6+0.45+0.45</f>
+        <v>1.5</v>
+      </c>
+      <c r="F46" s="33">
+        <v>0.1</v>
+      </c>
+      <c r="G46" s="33">
+        <f t="shared" si="15"/>
+        <v>-1.097226455348979</v>
+      </c>
+      <c r="H46" s="17"/>
+      <c r="I46" s="17"/>
+      <c r="J46" s="18"/>
+      <c r="K46" s="17"/>
+    </row>
+    <row r="47" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="2"/>
+      <c r="B47" s="40" t="s">
         <v>36</v>
       </c>
-      <c r="C46" s="3"/>
-      <c r="D46" s="4"/>
-      <c r="E46" s="5"/>
-      <c r="F46" s="5"/>
-      <c r="G46" s="39">
-        <f>SUM(G41:G45)</f>
-        <v>2.4063968411032794</v>
-      </c>
-      <c r="H46" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="I46" s="6">
+      <c r="C47" s="3"/>
+      <c r="D47" s="4"/>
+      <c r="E47" s="5"/>
+      <c r="F47" s="5"/>
+      <c r="G47" s="39">
+        <f>SUM(G43:G46)</f>
+        <v>2.0772289044985861</v>
+      </c>
+      <c r="H47" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="I47" s="6">
         <v>13351.1</v>
       </c>
-      <c r="J46" s="39">
-        <f>G46*I46</f>
-        <v>32128.044865253996</v>
-      </c>
-      <c r="K46" s="5"/>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A47" s="16"/>
-      <c r="B47" s="32" t="s">
-        <v>26</v>
-      </c>
-      <c r="C47" s="17"/>
-      <c r="D47" s="17"/>
-      <c r="E47" s="17"/>
-      <c r="F47" s="17"/>
-      <c r="G47" s="17"/>
-      <c r="H47" s="17"/>
-      <c r="I47" s="17"/>
-      <c r="J47" s="18">
-        <f>0.13*G46*4169.92</f>
-        <v>1304.4827010349404</v>
-      </c>
-      <c r="K47" s="17"/>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="J47" s="39">
+        <f>G47*I47</f>
+        <v>27733.290826851073</v>
+      </c>
+      <c r="K47" s="5"/>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="16"/>
       <c r="B48" s="32" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C48" s="17"/>
       <c r="D48" s="17"/>
@@ -2184,15 +2185,15 @@
       <c r="H48" s="17"/>
       <c r="I48" s="17"/>
       <c r="J48" s="18">
-        <f>0.13*G46*1414.16</f>
-        <v>442.39392038589983</v>
+        <f>0.13*G47*4169.92</f>
+        <v>1126.0441859480768</v>
       </c>
       <c r="K48" s="17"/>
     </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A49" s="16"/>
       <c r="B49" s="32" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C49" s="17"/>
       <c r="D49" s="17"/>
@@ -2202,15 +2203,15 @@
       <c r="H49" s="17"/>
       <c r="I49" s="17"/>
       <c r="J49" s="18">
-        <f>0.13*G46*(1652.5+737.97+349.56)</f>
-        <v>857.16793974866857</v>
+        <f>0.13*G47*1414.16</f>
+        <v>381.87942358614367</v>
       </c>
       <c r="K49" s="17"/>
     </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A50" s="16"/>
       <c r="B50" s="32" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C50" s="17"/>
       <c r="D50" s="17"/>
@@ -2220,14 +2221,16 @@
       <c r="H50" s="17"/>
       <c r="I50" s="17"/>
       <c r="J50" s="18">
-        <f>0.13*G46*42</f>
-        <v>13.138926752423908</v>
+        <f>0.13*G47*(1652.5+737.97+349.56)</f>
+        <v>739.91703697512401</v>
       </c>
       <c r="K50" s="17"/>
     </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A51" s="16"/>
-      <c r="B51" s="32"/>
+      <c r="B51" s="32" t="s">
+        <v>30</v>
+      </c>
       <c r="C51" s="17"/>
       <c r="D51" s="17"/>
       <c r="E51" s="17"/>
@@ -2235,16 +2238,15 @@
       <c r="G51" s="17"/>
       <c r="H51" s="17"/>
       <c r="I51" s="17"/>
-      <c r="J51" s="18"/>
+      <c r="J51" s="18">
+        <f>0.13*G47*42</f>
+        <v>11.341669818562281</v>
+      </c>
       <c r="K51" s="17"/>
     </row>
-    <row r="52" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A52" s="16">
-        <v>6</v>
-      </c>
-      <c r="B52" s="56" t="s">
-        <v>55</v>
-      </c>
+    <row r="52" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A52" s="16"/>
+      <c r="B52" s="32"/>
       <c r="C52" s="17"/>
       <c r="D52" s="17"/>
       <c r="E52" s="17"/>
@@ -2252,98 +2254,96 @@
       <c r="G52" s="17"/>
       <c r="H52" s="17"/>
       <c r="I52" s="17"/>
-      <c r="J52" s="17"/>
+      <c r="J52" s="18"/>
       <c r="K52" s="17"/>
     </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A53" s="16"/>
-      <c r="B53" s="32" t="s">
-        <v>46</v>
-      </c>
-      <c r="C53" s="17">
-        <f>C32</f>
-        <v>4</v>
-      </c>
-      <c r="D53" s="33">
-        <f>D32</f>
-        <v>3.6574215178299299</v>
-      </c>
-      <c r="E53" s="33">
-        <v>0.45</v>
-      </c>
-      <c r="F53" s="33">
-        <f>1.2</f>
-        <v>1.2</v>
-      </c>
-      <c r="G53" s="33">
-        <f>PRODUCT(C53:F53)</f>
-        <v>7.9000304785126483</v>
-      </c>
+    <row r="53" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A53" s="16">
+        <v>6</v>
+      </c>
+      <c r="B53" s="43" t="s">
+        <v>54</v>
+      </c>
+      <c r="C53" s="17"/>
+      <c r="D53" s="17"/>
+      <c r="E53" s="17"/>
+      <c r="F53" s="17"/>
+      <c r="G53" s="17"/>
       <c r="H53" s="17"/>
       <c r="I53" s="17"/>
       <c r="J53" s="17"/>
       <c r="K53" s="17"/>
-      <c r="M53" s="33">
+    </row>
+    <row r="54" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A54" s="16"/>
+      <c r="B54" s="32" t="s">
+        <v>45</v>
+      </c>
+      <c r="C54" s="17">
+        <f>2*2</f>
+        <v>4</v>
+      </c>
+      <c r="D54" s="33">
+        <f>8/3.281</f>
+        <v>2.4382810118866196</v>
+      </c>
+      <c r="E54" s="33">
+        <v>0.45</v>
+      </c>
+      <c r="F54" s="33">
+        <v>0.9</v>
+      </c>
+      <c r="G54" s="33">
+        <f>PRODUCT(C54:F54)</f>
+        <v>3.9500152392563237</v>
+      </c>
+      <c r="H54" s="17"/>
+      <c r="I54" s="17"/>
+      <c r="J54" s="17"/>
+      <c r="K54" s="17"/>
+      <c r="M54" s="33">
         <f>7</f>
         <v>7</v>
       </c>
-      <c r="N53" s="33">
+      <c r="N54" s="33">
         <f>2</f>
         <v>2</v>
       </c>
-      <c r="O53" s="33"/>
-      <c r="P53" s="33">
-        <f>PI()*M53*SQRT(M53^2+N53^2)</f>
+      <c r="O54" s="33"/>
+      <c r="P54" s="33">
+        <f>PI()*M54*SQRT(M54^2+N54^2)</f>
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="54" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="2"/>
-      <c r="B54" s="34" t="s">
+    <row r="55" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="2"/>
+      <c r="B55" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="C54" s="3"/>
-      <c r="D54" s="4"/>
-      <c r="E54" s="5"/>
-      <c r="F54" s="5"/>
-      <c r="G54" s="6">
-        <f>SUM(G53:G53)</f>
-        <v>7.9000304785126483</v>
-      </c>
-      <c r="H54" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="I54" s="6">
+      <c r="C55" s="3"/>
+      <c r="D55" s="4"/>
+      <c r="E55" s="5"/>
+      <c r="F55" s="5"/>
+      <c r="G55" s="6">
+        <f>SUM(G54:G54)</f>
+        <v>3.9500152392563237</v>
+      </c>
+      <c r="H55" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="I55" s="6">
         <v>6337.3</v>
       </c>
-      <c r="J54" s="18">
-        <f>G54*I54</f>
-        <v>50064.86315147821</v>
-      </c>
-      <c r="K54" s="5"/>
-    </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A55" s="16"/>
-      <c r="B55" s="32" t="s">
-        <v>52</v>
-      </c>
-      <c r="C55" s="17"/>
-      <c r="D55" s="17"/>
-      <c r="E55" s="17"/>
-      <c r="F55" s="17"/>
-      <c r="G55" s="17"/>
-      <c r="H55" s="17"/>
-      <c r="I55" s="17"/>
       <c r="J55" s="18">
-        <f>0.13*G54*2577.63</f>
-        <v>2647.2362231027128</v>
-      </c>
-      <c r="K55" s="17"/>
-    </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.3">
+        <f>G55*I55</f>
+        <v>25032.431575739101</v>
+      </c>
+      <c r="K55" s="5"/>
+    </row>
+    <row r="56" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56" s="16"/>
       <c r="B56" s="32" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C56" s="17"/>
       <c r="D56" s="17"/>
@@ -2353,15 +2353,15 @@
       <c r="H56" s="17"/>
       <c r="I56" s="17"/>
       <c r="J56" s="18">
-        <f>0.13*G54*257.76</f>
-        <v>264.7205412983846</v>
+        <f>0.13*G55*2577.63</f>
+        <v>1323.6181115513564</v>
       </c>
       <c r="K56" s="17"/>
     </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A57" s="16"/>
       <c r="B57" s="32" t="s">
-        <v>29</v>
+        <v>52</v>
       </c>
       <c r="C57" s="17"/>
       <c r="D57" s="17"/>
@@ -2371,15 +2371,15 @@
       <c r="H57" s="17"/>
       <c r="I57" s="17"/>
       <c r="J57" s="18">
-        <f>0.13*G54*133.56</f>
-        <v>137.1666491923194</v>
+        <f>0.13*G55*257.76</f>
+        <v>132.3602706491923</v>
       </c>
       <c r="K57" s="17"/>
     </row>
-    <row r="58" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A58" s="16"/>
       <c r="B58" s="32" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C58" s="17"/>
       <c r="D58" s="17"/>
@@ -2389,14 +2389,16 @@
       <c r="H58" s="17"/>
       <c r="I58" s="17"/>
       <c r="J58" s="18">
-        <f>0.13*G54*19.6</f>
-        <v>20.129277659250228</v>
+        <f>0.13*G55*133.56</f>
+        <v>68.583324596159699</v>
       </c>
       <c r="K58" s="17"/>
     </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A59" s="16"/>
-      <c r="B59" s="32"/>
+      <c r="B59" s="32" t="s">
+        <v>30</v>
+      </c>
       <c r="C59" s="17"/>
       <c r="D59" s="17"/>
       <c r="E59" s="17"/>
@@ -2404,222 +2406,187 @@
       <c r="G59" s="17"/>
       <c r="H59" s="17"/>
       <c r="I59" s="17"/>
-      <c r="J59" s="18"/>
+      <c r="J59" s="18">
+        <f>0.13*G55*19.6</f>
+        <v>10.064638829625114</v>
+      </c>
       <c r="K59" s="17"/>
     </row>
-    <row r="60" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="2">
+    <row r="60" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A60" s="16"/>
+      <c r="B60" s="32"/>
+      <c r="C60" s="17"/>
+      <c r="D60" s="17"/>
+      <c r="E60" s="17"/>
+      <c r="F60" s="17"/>
+      <c r="G60" s="17"/>
+      <c r="H60" s="17"/>
+      <c r="I60" s="17"/>
+      <c r="J60" s="18"/>
+      <c r="K60" s="17"/>
+    </row>
+    <row r="61" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="2">
         <v>7</v>
       </c>
-      <c r="B60" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C60" s="3">
-        <f>2*1</f>
-        <v>2</v>
-      </c>
-      <c r="D60" s="4"/>
-      <c r="E60" s="5"/>
-      <c r="F60" s="5"/>
-      <c r="G60" s="7">
-        <f t="shared" ref="G60" si="13">PRODUCT(C60:F60)</f>
-        <v>2</v>
-      </c>
-      <c r="H60" s="7" t="s">
+      <c r="B61" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C61" s="3">
+        <v>1</v>
+      </c>
+      <c r="D61" s="4"/>
+      <c r="E61" s="5"/>
+      <c r="F61" s="5"/>
+      <c r="G61" s="7">
+        <f t="shared" ref="G61" si="16">PRODUCT(C61:F61)</f>
+        <v>1</v>
+      </c>
+      <c r="H61" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I60" s="6">
-        <v>2500</v>
-      </c>
-      <c r="J60" s="7">
-        <f>G60*I60</f>
-        <v>5000</v>
-      </c>
-      <c r="K60" s="5"/>
-    </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A61" s="16"/>
-      <c r="B61" s="32"/>
-      <c r="C61" s="17"/>
-      <c r="D61" s="17"/>
-      <c r="E61" s="17"/>
-      <c r="F61" s="17"/>
-      <c r="G61" s="17"/>
-      <c r="H61" s="17"/>
-      <c r="I61" s="17"/>
-      <c r="J61" s="18"/>
-      <c r="K61" s="17"/>
-    </row>
-    <row r="62" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="2">
-        <v>8</v>
-      </c>
-      <c r="B62" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C62" s="3">
-        <v>1</v>
-      </c>
+      <c r="I61" s="6">
+        <v>1000</v>
+      </c>
+      <c r="J61" s="7">
+        <f>G61*I61</f>
+        <v>1000</v>
+      </c>
+      <c r="K61" s="5"/>
+    </row>
+    <row r="62" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A62" s="2"/>
+      <c r="B62" s="8"/>
+      <c r="C62" s="3"/>
       <c r="D62" s="4"/>
       <c r="E62" s="5"/>
       <c r="F62" s="5"/>
-      <c r="G62" s="7">
-        <f t="shared" ref="G62" si="14">PRODUCT(C62:F62)</f>
-        <v>1</v>
-      </c>
-      <c r="H62" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="I62" s="6">
-        <v>1000</v>
-      </c>
-      <c r="J62" s="7">
-        <f>G62*I62</f>
-        <v>1000</v>
-      </c>
+      <c r="G62" s="6"/>
+      <c r="H62" s="7"/>
+      <c r="I62" s="6"/>
+      <c r="J62" s="18"/>
       <c r="K62" s="5"/>
     </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A63" s="2"/>
-      <c r="B63" s="8"/>
-      <c r="C63" s="3"/>
-      <c r="D63" s="4"/>
-      <c r="E63" s="5"/>
-      <c r="F63" s="5"/>
-      <c r="G63" s="6"/>
-      <c r="H63" s="7"/>
-      <c r="I63" s="6"/>
-      <c r="J63" s="18"/>
-      <c r="K63" s="5"/>
-    </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A64" s="21"/>
-      <c r="B64" s="22" t="s">
+    <row r="63" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A63" s="21"/>
+      <c r="B63" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="C64" s="23"/>
-      <c r="D64" s="24"/>
-      <c r="E64" s="24"/>
-      <c r="F64" s="24"/>
-      <c r="G64" s="18"/>
-      <c r="H64" s="18"/>
-      <c r="I64" s="18"/>
-      <c r="J64" s="18">
-        <f>SUM(J9:J62)</f>
-        <v>223805.92450562009</v>
-      </c>
-      <c r="K64" s="25"/>
-    </row>
-    <row r="65" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="M65" s="20"/>
-      <c r="N65" s="20"/>
-      <c r="O65" s="20"/>
-      <c r="P65" s="20"/>
-      <c r="Q65" s="20"/>
-      <c r="R65" s="20"/>
-      <c r="S65" s="20"/>
-    </row>
-    <row r="66" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="26"/>
+      <c r="C63" s="23"/>
+      <c r="D63" s="24"/>
+      <c r="E63" s="24"/>
+      <c r="F63" s="24"/>
+      <c r="G63" s="18"/>
+      <c r="H63" s="18"/>
+      <c r="I63" s="18"/>
+      <c r="J63" s="18">
+        <f>SUM(J9:J61)</f>
+        <v>234835.07491669987</v>
+      </c>
+      <c r="K63" s="25"/>
+    </row>
+    <row r="64" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="M64" s="20"/>
+      <c r="N64" s="20"/>
+      <c r="O64" s="20"/>
+      <c r="P64" s="20"/>
+      <c r="Q64" s="20"/>
+      <c r="R64" s="20"/>
+      <c r="S64" s="20"/>
+    </row>
+    <row r="65" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="26"/>
+      <c r="B65" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="C65" s="44">
+        <f>J63</f>
+        <v>234835.07491669987</v>
+      </c>
+      <c r="D65" s="45"/>
+      <c r="E65" s="9">
+        <v>100</v>
+      </c>
+      <c r="F65" s="26"/>
+      <c r="G65" s="28"/>
+      <c r="H65" s="26"/>
+      <c r="I65" s="29"/>
+      <c r="J65" s="30"/>
+      <c r="K65" s="31"/>
+      <c r="M65" s="19"/>
+      <c r="N65" s="19"/>
+      <c r="O65" s="19"/>
+      <c r="P65" s="19"/>
+      <c r="Q65" s="19"/>
+      <c r="R65" s="19"/>
+      <c r="S65" s="19"/>
+    </row>
+    <row r="66" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B66" s="27" t="s">
-        <v>19</v>
-      </c>
-      <c r="C66" s="49">
-        <f>J64</f>
-        <v>223805.92450562009</v>
-      </c>
-      <c r="D66" s="50"/>
-      <c r="E66" s="9">
-        <v>100</v>
-      </c>
-      <c r="F66" s="26"/>
-      <c r="G66" s="28"/>
-      <c r="H66" s="26"/>
-      <c r="I66" s="29"/>
-      <c r="J66" s="30"/>
-      <c r="K66" s="31"/>
-      <c r="M66" s="19"/>
-      <c r="N66" s="19"/>
-      <c r="O66" s="19"/>
-      <c r="P66" s="19"/>
-      <c r="Q66" s="19"/>
-      <c r="R66" s="19"/>
-      <c r="S66" s="19"/>
-    </row>
-    <row r="67" spans="1:19" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+      <c r="C66" s="48">
+        <v>200000</v>
+      </c>
+      <c r="D66" s="49"/>
+      <c r="E66" s="9"/>
+    </row>
+    <row r="67" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B67" s="27" t="s">
-        <v>21</v>
-      </c>
-      <c r="C67" s="53">
-        <v>200000</v>
-      </c>
-      <c r="D67" s="54"/>
-      <c r="E67" s="9"/>
-    </row>
-    <row r="68" spans="1:19" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+      <c r="C67" s="48">
+        <f>C66-C69-C70</f>
+        <v>190000</v>
+      </c>
+      <c r="D67" s="49"/>
+      <c r="E67" s="9">
+        <f>C67/C65*100</f>
+        <v>80.907845673137345</v>
+      </c>
+    </row>
+    <row r="68" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B68" s="27" t="s">
-        <v>22</v>
-      </c>
-      <c r="C68" s="53">
-        <f>C67-C70-C71</f>
-        <v>190000</v>
-      </c>
-      <c r="D68" s="54"/>
+        <v>31</v>
+      </c>
+      <c r="C68" s="50">
+        <f>C65-C67</f>
+        <v>44835.074916699872</v>
+      </c>
+      <c r="D68" s="50"/>
       <c r="E68" s="9">
-        <f>C68/C66*100</f>
-        <v>84.894982302056448</v>
-      </c>
-    </row>
-    <row r="69" spans="1:19" x14ac:dyDescent="0.3">
+        <f>100-E67</f>
+        <v>19.092154326862655</v>
+      </c>
+    </row>
+    <row r="69" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B69" s="27" t="s">
-        <v>31</v>
-      </c>
-      <c r="C69" s="55">
-        <f>C66-C68</f>
-        <v>33805.924505620089</v>
-      </c>
-      <c r="D69" s="55"/>
+        <v>23</v>
+      </c>
+      <c r="C69" s="44">
+        <f>C66*0.03</f>
+        <v>6000</v>
+      </c>
+      <c r="D69" s="45"/>
       <c r="E69" s="9">
-        <f>100-E68</f>
-        <v>15.105017697943552</v>
-      </c>
-    </row>
-    <row r="70" spans="1:19" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="70" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B70" s="27" t="s">
-        <v>23</v>
-      </c>
-      <c r="C70" s="49">
-        <f>C67*0.03</f>
-        <v>6000</v>
-      </c>
-      <c r="D70" s="50"/>
+        <v>24</v>
+      </c>
+      <c r="C70" s="44">
+        <f>C66*0.02</f>
+        <v>4000</v>
+      </c>
+      <c r="D70" s="45"/>
       <c r="E70" s="9">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="71" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="B71" s="27" t="s">
-        <v>24</v>
-      </c>
-      <c r="C71" s="49">
-        <f>C67*0.02</f>
-        <v>4000</v>
-      </c>
-      <c r="D71" s="50"/>
-      <c r="E71" s="9">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="C70:D70"/>
-    <mergeCell ref="C71:D71"/>
-    <mergeCell ref="A7:F7"/>
-    <mergeCell ref="H7:K7"/>
-    <mergeCell ref="C66:D66"/>
-    <mergeCell ref="C67:D67"/>
-    <mergeCell ref="C68:D68"/>
-    <mergeCell ref="C69:D69"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="H6:K6"/>
     <mergeCell ref="A1:K1"/>
@@ -2627,11 +2594,22 @@
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A5:K5"/>
+    <mergeCell ref="C69:D69"/>
+    <mergeCell ref="C70:D70"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="H7:K7"/>
+    <mergeCell ref="C65:D65"/>
+    <mergeCell ref="C66:D66"/>
+    <mergeCell ref="C67:D67"/>
+    <mergeCell ref="C68:D68"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
   <headerFooter>
     <oddFooter>&amp;LPrepared By:&amp;CChecked By:&amp;RApproved By:</oddFooter>
   </headerFooter>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="45" max="10" man="1"/>
+  </rowBreaks>
 </worksheet>
 </file>
</xml_diff>